<commit_message>
Add individual student dashboard and profile view
</commit_message>
<xml_diff>
--- a/reports/students_data.xlsx
+++ b/reports/students_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -603,123 +603,123 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ayan</t>
+          <t>asif</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ayan@gmail.com</t>
+          <t>asif@gmail.com</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>03000000002</t>
+          <t>03000000012</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Software Engineering</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G5" t="n">
-        <v>3.95</v>
-      </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
+        <v>3.67</v>
+      </c>
+      <c r="H5" t="n">
+        <v>82.75</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>{}</t>
+          <t>{"Web Tech": 88.0, "Networking": 67.0, "Cyber Security": 77.0, "Cloud Computing": 99.0}</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>moiz</t>
+          <t>ayan</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>moiz@gmail.com</t>
+          <t>ayan@gmail.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>03000000008</t>
+          <t>03000000002</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Computer Science</t>
+          <t>Software Engineering</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G6" t="n">
-        <v>3.77</v>
-      </c>
-      <c r="H6" t="n">
-        <v>76.83</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
+        <v>3.95</v>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
-          <t>{"DLD": 66.0, "DBMS": 77.0, "Python": 88.0, "Calculus": 87.0, "Statistics": 76.0, "Mathematics": 67.0}</t>
+          <t>{}</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>muzammil</t>
+          <t>moiz</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>muzammil@gmail.com</t>
+          <t>moiz@gmail.com</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>03000000005</t>
+          <t>03000000008</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Computer Science</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G7" t="n">
-        <v>3.04</v>
+        <v>3.77</v>
       </c>
       <c r="H7" t="n">
-        <v>70.17</v>
+        <v>76.83</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -728,121 +728,121 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>{"DLD": 89.0, "DBMS": 56.0, "Python": 67.0, "Calculus": 55.0, "Statistics": 88.0, "Mathematics": 66.0}</t>
+          <t>{"DLD": 66.0, "DBMS": 77.0, "Python": 88.0, "Calculus": 87.0, "Statistics": 76.0, "Mathematics": 67.0}</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>rehan</t>
+          <t>muzammil</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>rehan@gmail.com</t>
+          <t>muzammil@gmail.com</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>03000000001</t>
+          <t>03000000005</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Computer Science</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G8" t="n">
-        <v>3.38</v>
+        <v>3.04</v>
       </c>
       <c r="H8" t="n">
-        <v>81.17</v>
+        <v>70.17</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>{"DLD": 88.0, "DBMS": 88.0, "Python": 77.0, "Calculus": 67.0, "Statistics": 78.0, "Mathematics": 89.0}</t>
+          <t>{"DLD": 89.0, "DBMS": 56.0, "Python": 67.0, "Calculus": 55.0, "Statistics": 88.0, "Mathematics": 66.0}</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>sameer</t>
+          <t>rehan</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>sameer@gmail.com</t>
+          <t>rehan@gmail.com</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>03000000007</t>
+          <t>03000000001</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Data Science</t>
+          <t>Computer Science</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G9" t="n">
-        <v>3.64</v>
+        <v>3.38</v>
       </c>
       <c r="H9" t="n">
-        <v>73.67</v>
+        <v>81.17</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>{"DLD": 56.0, "DBMS": 78.0, "Python": 88.0, "Calculus": 76.0, "Statistics": 77.0, "Mathematics": 67.0}</t>
+          <t>{"DLD": 88.0, "DBMS": 88.0, "Python": 77.0, "Calculus": 67.0, "Statistics": 78.0, "Mathematics": 89.0}</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ukasha</t>
+          <t>sameer</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ukasha@gmail.com</t>
+          <t>sameer@gmail.com</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>03000000004</t>
+          <t>03000000007</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -854,103 +854,201 @@
         <v>3</v>
       </c>
       <c r="G10" t="n">
-        <v>3.62</v>
-      </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
+        <v>3.64</v>
+      </c>
+      <c r="H10" t="n">
+        <v>73.67</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>{}</t>
+          <t>{"DLD": 56.0, "DBMS": 78.0, "Python": 88.0, "Calculus": 76.0, "Statistics": 77.0, "Mathematics": 67.0}</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>uzair</t>
+          <t>sohaib</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>uzair@gmail.com</t>
+          <t>sohaib@gmail.com</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>03000000000</t>
+          <t>03000000011</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Data Science</t>
+          <t>Software Engineering</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G11" t="n">
-        <v>3.57</v>
+        <v>3.11</v>
       </c>
       <c r="H11" t="n">
-        <v>91.17</v>
+        <v>74</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>A+</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>{"DLD": 92.0, "DBMS": 87.0, "Python": 89.0, "Calculus": 80.0, "Statistics": 99.0, "Mathematics": 100.0}</t>
+          <t>{"SQA": 77.0, "DBMS": 76.0, "Software Design": 56.0, "Web Engineering": 87.0}</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>waqas</t>
+          <t>ukasha</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>waqas@gmail.com</t>
+          <t>ukasha@gmail.com</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>03000000009</t>
+          <t>03000000004</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Software Engineering</t>
+          <t>Data Science</t>
         </is>
       </c>
       <c r="F12" t="n">
         <v>3</v>
       </c>
       <c r="G12" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="H12" t="n">
+        <v>72.25</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>{"Python": 66.0, "Statistics": 79.0, "Linear Algebra": 78.0, "Machine Learning": 66.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>uzair</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>uzair@gmail.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>03000000000</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>3</v>
+      </c>
+      <c r="G13" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="H13" t="n">
+        <v>91.17</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>{"DLD": 92.0, "DBMS": 87.0, "Python": 89.0, "Calculus": 80.0, "Statistics": 99.0, "Mathematics": 100.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>waqas</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>waqas@gmail.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>03000000009</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Software Engineering</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>3</v>
+      </c>
+      <c r="G14" t="n">
         <v>3.31</v>
       </c>
-      <c r="H12" t="n">
+      <c r="H14" t="n">
         <v>61.17</v>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>{"DLD": 77.0, "DBMS": 65.0, "Python": 66.0, "Calculus": 54.0, "Statistics": 55.0, "Mathematics": 50.0}</t>
         </is>

</xml_diff>